<commit_message>
adjusted positions of some components created output job filds
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_current_measurement_hc5fw/01/BOM/BOM_JLC-uz_per_current_measurement_hc5fw.xlsx
+++ b/Project Outputs for uz_per_current_measurement_hc5fw/01/BOM/BOM_JLC-uz_per_current_measurement_hc5fw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_per_current_measurement_hc5fw\Project Outputs for uz_per_current_measurement_hc5fw\01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61B6ABC6-01B2-4C3A-BC8E-3D5477BDCBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9F11C6D-F177-4202-BE9E-506706F6C025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26025" yWindow="3015" windowWidth="24000" windowHeight="16980" xr2:uid="{8D10F421-1E0E-4F30-A478-44687F4D7F25}"/>
+    <workbookView xWindow="26025" yWindow="3015" windowWidth="24000" windowHeight="16980" xr2:uid="{812DBA70-BB8D-433B-AC39-181471FFF942}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_current_measurem" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="191">
   <si>
     <t>Quantity</t>
   </si>
@@ -579,10 +579,10 @@
     <t>U4A, U4B, U4C, U4D</t>
   </si>
   <si>
-    <t>145MHz 240uV 700nA Single Channel 95MHz SOIC-8 Differential Amplifiers ROHS</t>
-  </si>
-  <si>
-    <t>ADA4940-1ARZ-R7</t>
+    <t>THS452x Very Low Power, Negative Rail Input, Rail-To-Rail Output, Fully Differential Amplifier</t>
+  </si>
+  <si>
+    <t>SOIC127P600X175-8N</t>
   </si>
   <si>
     <t>THS4521IDR</t>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7B7F79-38DE-44BF-9204-2F6F1B2B4F70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E2E48F-7992-4EC3-A219-87F48B6E8A1B}">
   <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1885,7 +1885,9 @@
       <c r="D29" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E29" s="1"/>
+      <c r="E29" s="2" t="s">
+        <v>177</v>
+      </c>
       <c r="F29" s="2" t="s">
         <v>179</v>
       </c>

</xml_diff>

<commit_message>
Erdung von RJ45 Buchse über Widerstand und Kapazität parallel umgesetzt Output Job neu erstellt
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_current_measurement_hc5fw/01/BOM/BOM_JLC-uz_per_current_measurement_hc5fw.xlsx
+++ b/Project Outputs for uz_per_current_measurement_hc5fw/01/BOM/BOM_JLC-uz_per_current_measurement_hc5fw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_per_current_measurement_hc5fw\Project Outputs for uz_per_current_measurement_hc5fw\01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{766B6546-BF92-44B6-AC0B-F3E34BEEC603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5148561F-9C04-4D1B-A8AC-9B13C85564C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26025" yWindow="3015" windowWidth="24000" windowHeight="16980" xr2:uid="{CC30DD20-B079-4E22-8BB2-22440D8C453E}"/>
+    <workbookView xWindow="26025" yWindow="3015" windowWidth="24000" windowHeight="16980" xr2:uid="{72709656-1F20-427F-8A8E-53B14E3AE6E6}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_current_measurem" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="197">
   <si>
     <t>Quantity</t>
   </si>
@@ -258,6 +258,24 @@
     <t>C1622</t>
   </si>
   <si>
+    <t>100pF</t>
+  </si>
+  <si>
+    <t>C54</t>
+  </si>
+  <si>
+    <t>100pF 1kV C0G ±5% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+  </si>
+  <si>
+    <t>C_1206_TE</t>
+  </si>
+  <si>
+    <t>1206CG101J102NT</t>
+  </si>
+  <si>
+    <t>C9188</t>
+  </si>
+  <si>
     <t>KT-0603R</t>
   </si>
   <si>
@@ -496,6 +514,21 @@
   </si>
   <si>
     <t>C114625</t>
+  </si>
+  <si>
+    <t>1M</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>Vishay / Dale</t>
+  </si>
+  <si>
+    <t>CRCW06031M00FKEAC</t>
+  </si>
+  <si>
+    <t>C844537</t>
   </si>
   <si>
     <t>TPSM365R6</t>
@@ -973,8 +1006,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A848E61-2347-4728-BD30-5F9D846F5E55}">
-  <dimension ref="A1:K30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E46A0352-5FD3-421C-A81B-4A7F83676EEE}">
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -1336,7 +1369,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>72</v>
@@ -1345,19 +1378,21 @@
         <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>77</v>
@@ -1365,7 +1400,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>78</v>
@@ -1376,9 +1411,7 @@
       <c r="D13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="E13" s="1"/>
       <c r="F13" s="2" t="s">
         <v>81</v>
       </c>
@@ -1388,44 +1421,46 @@
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="K14" s="1"/>
+        <v>89</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>91</v>
@@ -1437,100 +1472,98 @@
         <v>93</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>95</v>
-      </c>
+      <c r="K15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>113</v>
@@ -1541,64 +1574,64 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="F20" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1611,7 +1644,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>128</v>
@@ -1629,46 +1662,46 @@
         <v>131</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>137</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1676,30 +1709,30 @@
         <v>8</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="G23" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1707,61 +1740,61 @@
         <v>8</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>155</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1769,30 +1802,30 @@
         <v>1</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="E26" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>162</v>
+        <v>119</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>163</v>
+        <v>120</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1800,121 +1833,183 @@
         <v>1</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="E27" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>172</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>175</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="G29" s="2" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E30" s="1"/>
       <c r="F30" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>4</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>2</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>